<commit_message>
reworked Rev01b to Rev02b, generated output files. Changes: - increased clearances between phase connectors in order to provide enough clearance for about 250V - added connections on DSUB9 connector in order to support both uz_d_resolver, and uz_d_absolute_encoder PCBs
</commit_message>
<xml_diff>
--- a/Project Outputs for UZ_PER_deskbench_terminal/Rev01b/BOM/BOM_JLC-UZ_PER_deskbench_terminal.xlsx
+++ b/Project Outputs for UZ_PER_deskbench_terminal/Rev01b/BOM/BOM_JLC-UZ_PER_deskbench_terminal.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\UltraZohm\uz_per_deskbench_terminal\Project Outputs for UZ_PER_deskbench_terminal\Rev01b\BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_per_deskbench_terminal\Project Outputs for UZ_PER_deskbench_terminal\Rev01b\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C17F35FC-9730-49DD-9802-D5F70AB85350}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37952E33-12F5-473A-88EA-055C7F59B5AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-29220" yWindow="1500" windowWidth="23040" windowHeight="12120" xr2:uid="{8C88FD5C-07CD-43B8-94BE-D97FB9498931}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{8C88FD5C-07CD-43B8-94BE-D97FB9498931}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM_JLC-UZ_PER_deskbench_termin" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="43">
   <si>
     <t>Quantity</t>
   </si>
@@ -159,6 +159,15 @@
   </si>
   <si>
     <t>Serial Number</t>
+  </si>
+  <si>
+    <t>C7437327</t>
+  </si>
+  <si>
+    <t>in our stock</t>
+  </si>
+  <si>
+    <t>GlobalSourcingMouser</t>
   </si>
 </sst>
 </file>
@@ -174,7 +183,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -184,6 +193,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD3D3D3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -215,12 +236,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -239,9 +263,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -279,7 +303,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -385,7 +409,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -527,7 +551,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -535,22 +559,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3DBF90B-AB4F-4B26-B0C7-40C9D23F47C1}">
-  <dimension ref="A1:K8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:L8"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" customWidth="1"/>
-    <col min="2" max="2" width="18.77734375" customWidth="1"/>
-    <col min="3" max="3" width="17.44140625" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" customWidth="1"/>
-    <col min="5" max="5" width="16.6640625" customWidth="1"/>
-    <col min="6" max="6" width="16.21875" customWidth="1"/>
-    <col min="7" max="7" width="23.88671875" customWidth="1"/>
-    <col min="8" max="8" width="8.6640625" customWidth="1"/>
+    <col min="1" max="1" width="9.453125" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" customWidth="1"/>
+    <col min="3" max="3" width="17.453125" customWidth="1"/>
+    <col min="4" max="4" width="16.36328125" customWidth="1"/>
+    <col min="5" max="5" width="16.6328125" customWidth="1"/>
+    <col min="6" max="6" width="16.1796875" customWidth="1"/>
+    <col min="7" max="7" width="23.90625" customWidth="1"/>
+    <col min="8" max="8" width="8.6328125" customWidth="1"/>
     <col min="9" max="9" width="10" customWidth="1"/>
-    <col min="10" max="11" width="16.33203125" customWidth="1"/>
+    <col min="10" max="11" width="16.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -584,8 +608,11 @@
       <c r="K1" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="4" t="s">
+        <v>1</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -612,9 +639,14 @@
       <c r="J2" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K2" s="1"/>
+      <c r="K2" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="L2" t="s">
+        <v>41</v>
+      </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -641,9 +673,14 @@
       <c r="J3" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K3" s="1"/>
+      <c r="K3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="L3" t="s">
+        <v>41</v>
+      </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>1</v>
       </c>
@@ -670,9 +707,14 @@
       <c r="J4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="1"/>
+      <c r="K4" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="L4" t="s">
+        <v>41</v>
+      </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>1</v>
       </c>
@@ -697,11 +739,14 @@
       <c r="J5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="K5" s="2" t="s">
+      <c r="K5" s="6" t="s">
         <v>26</v>
       </c>
+      <c r="L5" t="s">
+        <v>41</v>
+      </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>1</v>
       </c>
@@ -726,9 +771,12 @@
       <c r="J6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="K6" s="1"/>
+      <c r="K6" s="7"/>
+      <c r="L6" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>1</v>
       </c>
@@ -753,9 +801,12 @@
       <c r="J7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="K7" s="1"/>
+      <c r="K7" s="7"/>
+      <c r="L7" t="s">
+        <v>42</v>
+      </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>1</v>
       </c>

</xml_diff>